<commit_message>
Stage 8 review fixes: F-010
</commit_message>
<xml_diff>
--- a/output/archive/DurnesswickData/TechTransfer/NM12/Dosing/Bench_Sheets/NM12_dilution-check_092820_LP.xlsx
+++ b/output/archive/DurnesswickData/TechTransfer/NM12/Dosing/Bench_Sheets/NM12_dilution-check_092820_LP.xlsx
@@ -900,7 +900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -912,160 +912,55 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Dilution challenge, cosolvent-rich vehicle and dispersed alternative</t>
+          <t>Dilution challenge: development outcome</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Each vehicle loaded at dosing strength, then diluted into simulated gastric medium at the ratios below. Read by eye and by light microscopy at 0.5 h, 2 h and 24 h.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Undiluted screen</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>PEG400/water was clear and stable in the initial screen; this did not establish dilution stability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Dilution outcome</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>The cosolvent-rich vehicle failed the dilution challenge. Refer to the dilution bench records for vehicle identity, concentration, dilution ratios and observations.</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Vehicle</t>
+          <t>Selected approach</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Dilution ratio</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Precipitate seen</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Comment</t>
+          <t>Nimbravelle selected dispersed dosing. Refer to the selected recipe card for composition.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>PEG400/water 30:70 (cosolvent-rich)</t>
+          <t>Limitation</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>1:10</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Yes, within 0.5 h</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Fails. Drug falls out as needles</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>PEG400/water 30:70 (cosolvent-rich)</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>1:50</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Yes, within 0.5 h</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Fails at the higher ratio too</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>0.5% HPMC / 0.1% Tween 80 (dispersed)</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>1:10</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Redispersed cleanly after gentle inversion</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>0.5% HPMC / 0.1% Tween 80 (dispersed)</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>1:50</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Clean at 24 h</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>pH 4 citrate buffer</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>1:10</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Trace at 24 h</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Acceptable but not chosen</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Screen suitability</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Reference standard run before each dilution series. Passed.</t>
+          <t>The undiluted table is not evidence of absence of precipitation after dilution.</t>
         </is>
       </c>
     </row>
@@ -1107,24 +1002,24 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>08/17/2020</t>
+          <t>09/28/2020</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Interim: the cosolvent-rich vehicle has high equilibrium solubility, but it does not survive dilution. Dispersed options are the way forward for the dosing solution.</t>
+          <t>Final. Nimbravelle selected dispersed dosing after the cosolvent-rich vehicle failed dilution.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>08/24/2020</t>
+          <t>09/28/2020</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Pharmacy handling check with the client's clinical supplies team. Dispersed vehicle needs a shake step before each dose. Written into the dosing instructions.</t>
+          <t>Redispersion and withdrawal controls must accompany the dosing recipe. Re-establish uniform dispersion before withdrawal and follow the source handling instructions; settling can change the dose withdrawn.</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1031,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Final. Client selected the dispersed approach. Tradeoff accepted: a shake step on every dose in exchange for no precipitation on dilution.</t>
+          <t>The HPMC/Tween screen showed crystal growth, and citrate buffer showed caking at 24 h. These rows do not establish clean diluted preparations.</t>
         </is>
       </c>
     </row>

</xml_diff>